<commit_message>
Use Profit or loss in accrual and prepayment ledgers and add the 4 steps
The Chapter 11 ledger accounts, and the insurance account in the mock
test, now post to Profit or loss instead of Income statement. The notes,
revision sheet and Chapter 11 worked tabs explain how to write these
accounts in 4 steps: start of year (Balance b/d), Bank, Profit or Loss,
end of year (Balance c/d).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Cg2FRYV2NgKh9WWDoLcpR2
</commit_message>
<xml_diff>
--- a/excel/Mock_Test.xlsx
+++ b/excel/Mock_Test.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="284">
   <si>
     <t xml:space="preserve">Mock Test: Senior 1 Accounting (2 hours, 100 marks)</t>
   </si>
@@ -592,6 +592,9 @@
   </si>
   <si>
     <t xml:space="preserve">Balance b/d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit or loss</t>
   </si>
   <si>
     <t xml:space="preserve">Apr 1</t>
@@ -2714,7 +2717,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2749,7 +2752,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -2784,7 +2787,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -3848,7 +3851,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3883,7 +3886,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -3918,7 +3921,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -4711,7 +4714,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -4746,7 +4749,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -4781,7 +4784,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -5470,7 +5473,7 @@
       <c r="S26" s="50"/>
       <c r="T26" s="50"/>
       <c r="U26" s="38" t="s">
-        <v>128</v>
+        <v>181</v>
       </c>
       <c r="V26" s="38"/>
       <c r="W26" s="38"/>
@@ -5490,7 +5493,7 @@
     </row>
     <row r="27" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -5518,7 +5521,7 @@
       <c r="S27" s="50"/>
       <c r="T27" s="50"/>
       <c r="U27" s="38" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="V27" s="38"/>
       <c r="W27" s="38"/>
@@ -5583,7 +5586,7 @@
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -5756,7 +5759,7 @@
       <c r="C37" s="36"/>
       <c r="D37" s="36"/>
       <c r="E37" s="38" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F37" s="38"/>
       <c r="G37" s="38"/>
@@ -5785,7 +5788,7 @@
       <c r="C38" s="36"/>
       <c r="D38" s="36"/>
       <c r="E38" s="37" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F38" s="37"/>
       <c r="G38" s="37"/>
@@ -5805,7 +5808,7 @@
       <c r="C39" s="36"/>
       <c r="D39" s="36"/>
       <c r="E39" s="38" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F39" s="38"/>
       <c r="G39" s="38"/>
@@ -5944,7 +5947,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -5979,7 +5982,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -6014,7 +6017,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -6049,7 +6052,7 @@
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -6084,7 +6087,7 @@
     </row>
     <row r="7" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C7" s="20"/>
       <c r="D7" s="20"/>
@@ -6118,7 +6121,7 @@
     </row>
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="20" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C8" s="20"/>
       <c r="D8" s="20"/>
@@ -6152,7 +6155,7 @@
     </row>
     <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="20" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C9" s="20"/>
       <c r="D9" s="20"/>
@@ -6186,7 +6189,7 @@
     </row>
     <row r="10" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="20" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
@@ -6220,7 +6223,7 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -6289,7 +6292,7 @@
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
@@ -6324,7 +6327,7 @@
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -6359,7 +6362,7 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
@@ -6394,7 +6397,7 @@
     </row>
     <row r="18" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C18" s="20"/>
       <c r="D18" s="20"/>
@@ -6428,7 +6431,7 @@
     </row>
     <row r="19" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="20" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C19" s="20"/>
       <c r="D19" s="20"/>
@@ -6462,7 +6465,7 @@
     </row>
     <row r="20" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
@@ -6496,7 +6499,7 @@
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -6531,7 +6534,7 @@
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="64" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C23" s="64"/>
       <c r="D23" s="64"/>
@@ -6695,7 +6698,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -6730,7 +6733,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -6765,7 +6768,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -6800,7 +6803,7 @@
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -6835,7 +6838,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="34" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C6" s="34"/>
       <c r="D6" s="34"/>
@@ -6891,7 +6894,7 @@
       <c r="S7" s="23"/>
       <c r="T7" s="23"/>
       <c r="U7" s="24" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="V7" s="24"/>
       <c r="W7" s="24"/>
@@ -6899,7 +6902,7 @@
       <c r="Y7" s="24"/>
       <c r="Z7" s="24"/>
       <c r="AA7" s="24" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AB7" s="24"/>
       <c r="AC7" s="24"/>
@@ -6909,7 +6912,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="30" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C8" s="30"/>
       <c r="D8" s="30"/>
@@ -6947,7 +6950,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="30" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C9" s="30"/>
       <c r="D9" s="30"/>
@@ -6985,7 +6988,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="30" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
@@ -7023,7 +7026,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="30" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
@@ -7061,7 +7064,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="30" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -7099,7 +7102,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="30"/>
@@ -7137,7 +7140,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="30" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C14" s="30"/>
       <c r="D14" s="30"/>
@@ -7175,7 +7178,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="30" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C15" s="30"/>
       <c r="D15" s="30"/>
@@ -7213,7 +7216,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="30"/>
@@ -7251,7 +7254,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -7289,7 +7292,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="30" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
@@ -7327,7 +7330,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="30" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
@@ -7365,7 +7368,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="30" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
@@ -7403,7 +7406,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="30" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
@@ -7479,7 +7482,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="30" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
@@ -7517,7 +7520,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="30" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
@@ -7555,7 +7558,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="30" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C25" s="30"/>
       <c r="D25" s="30"/>
@@ -7593,7 +7596,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="30" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C26" s="30"/>
       <c r="D26" s="30"/>
@@ -7631,7 +7634,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="30" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -7745,7 +7748,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C30" s="30"/>
       <c r="D30" s="30"/>
@@ -7783,7 +7786,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C31" s="30"/>
       <c r="D31" s="30"/>
@@ -7821,7 +7824,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C32" s="30"/>
       <c r="D32" s="30"/>
@@ -7859,7 +7862,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="30" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C33" s="30"/>
       <c r="D33" s="30"/>
@@ -7897,7 +7900,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="30" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C34" s="30"/>
       <c r="D34" s="30"/>
@@ -7935,7 +7938,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="30" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C35" s="30"/>
       <c r="D35" s="30"/>
@@ -8014,7 +8017,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C38" s="23"/>
       <c r="D38" s="23"/>
@@ -8048,7 +8051,7 @@
     </row>
     <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
@@ -8083,7 +8086,7 @@
     </row>
     <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
@@ -8118,7 +8121,7 @@
     </row>
     <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
@@ -8153,7 +8156,7 @@
     </row>
     <row r="42" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C42" s="12"/>
       <c r="D42" s="12"/>
@@ -8188,7 +8191,7 @@
     </row>
     <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="12" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
@@ -8223,7 +8226,7 @@
     </row>
     <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C44" s="12"/>
       <c r="D44" s="12"/>
@@ -8258,7 +8261,7 @@
     </row>
     <row r="45" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="12"/>
@@ -8293,7 +8296,7 @@
     </row>
     <row r="46" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="12" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="12"/>
@@ -8328,7 +8331,7 @@
     </row>
     <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C47" s="12"/>
       <c r="D47" s="12"/>
@@ -8363,7 +8366,7 @@
     </row>
     <row r="49" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
@@ -8398,7 +8401,7 @@
     </row>
     <row r="51" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -8433,7 +8436,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="34" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C52" s="34"/>
       <c r="D52" s="34"/>
@@ -8468,7 +8471,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="34" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C53" s="34"/>
       <c r="D53" s="34"/>
@@ -8547,7 +8550,7 @@
       <c r="C55" s="36"/>
       <c r="D55" s="36"/>
       <c r="E55" s="38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F55" s="38"/>
       <c r="G55" s="38"/>
@@ -8576,7 +8579,7 @@
       <c r="C56" s="36"/>
       <c r="D56" s="36"/>
       <c r="E56" s="38" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F56" s="38"/>
       <c r="G56" s="38"/>
@@ -8603,7 +8606,7 @@
       <c r="C57" s="36"/>
       <c r="D57" s="36"/>
       <c r="E57" s="38" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F57" s="38"/>
       <c r="G57" s="38"/>
@@ -8632,7 +8635,7 @@
       <c r="C58" s="36"/>
       <c r="D58" s="36"/>
       <c r="E58" s="37" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F58" s="37"/>
       <c r="G58" s="37"/>
@@ -8652,7 +8655,7 @@
       <c r="C59" s="36"/>
       <c r="D59" s="36"/>
       <c r="E59" s="38" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F59" s="38"/>
       <c r="G59" s="38"/>
@@ -8676,12 +8679,12 @@
     </row>
     <row r="60" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C60" s="36"/>
       <c r="D60" s="36"/>
       <c r="E60" s="38" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F60" s="38"/>
       <c r="G60" s="38"/>
@@ -8710,7 +8713,7 @@
       <c r="C61" s="36"/>
       <c r="D61" s="36"/>
       <c r="E61" s="38" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F61" s="38"/>
       <c r="G61" s="38"/>
@@ -8734,12 +8737,12 @@
     </row>
     <row r="62" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C62" s="36"/>
       <c r="D62" s="36"/>
       <c r="E62" s="38" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F62" s="38"/>
       <c r="G62" s="38"/>
@@ -8773,7 +8776,7 @@
       <c r="C63" s="36"/>
       <c r="D63" s="36"/>
       <c r="E63" s="38" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F63" s="38"/>
       <c r="G63" s="38"/>
@@ -8802,7 +8805,7 @@
       <c r="C64" s="36"/>
       <c r="D64" s="36"/>
       <c r="E64" s="38" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F64" s="38"/>
       <c r="G64" s="38"/>
@@ -8836,7 +8839,7 @@
       <c r="C65" s="36"/>
       <c r="D65" s="36"/>
       <c r="E65" s="56" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F65" s="56"/>
       <c r="G65" s="56"/>
@@ -8860,12 +8863,12 @@
     </row>
     <row r="66" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C66" s="36"/>
       <c r="D66" s="36"/>
       <c r="E66" s="37" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F66" s="37"/>
       <c r="G66" s="37"/>
@@ -8885,7 +8888,7 @@
       <c r="C67" s="36"/>
       <c r="D67" s="36"/>
       <c r="E67" s="38" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F67" s="38"/>
       <c r="G67" s="38"/>
@@ -8912,7 +8915,7 @@
       <c r="C68" s="36"/>
       <c r="D68" s="36"/>
       <c r="E68" s="38" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F68" s="38"/>
       <c r="G68" s="38"/>
@@ -8973,7 +8976,7 @@
       <c r="C70" s="36"/>
       <c r="D70" s="36"/>
       <c r="E70" s="37" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F70" s="37"/>
       <c r="G70" s="37"/>
@@ -8993,7 +8996,7 @@
       <c r="C71" s="36"/>
       <c r="D71" s="36"/>
       <c r="E71" s="38" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F71" s="38"/>
       <c r="G71" s="38"/>
@@ -9020,7 +9023,7 @@
       <c r="C72" s="36"/>
       <c r="D72" s="36"/>
       <c r="E72" s="38" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F72" s="38"/>
       <c r="G72" s="38"/>
@@ -9047,7 +9050,7 @@
       <c r="C73" s="36"/>
       <c r="D73" s="36"/>
       <c r="E73" s="38" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F73" s="38"/>
       <c r="G73" s="38"/>
@@ -9074,7 +9077,7 @@
       <c r="C74" s="36"/>
       <c r="D74" s="36"/>
       <c r="E74" s="38" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F74" s="38"/>
       <c r="G74" s="38"/>
@@ -9101,7 +9104,7 @@
       <c r="C75" s="36"/>
       <c r="D75" s="36"/>
       <c r="E75" s="38" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F75" s="38"/>
       <c r="G75" s="38"/>
@@ -9128,7 +9131,7 @@
       <c r="C76" s="36"/>
       <c r="D76" s="36"/>
       <c r="E76" s="38" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F76" s="38"/>
       <c r="G76" s="38"/>
@@ -9182,7 +9185,7 @@
       <c r="C78" s="36"/>
       <c r="D78" s="36"/>
       <c r="E78" s="38" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F78" s="38"/>
       <c r="G78" s="38"/>
@@ -9209,7 +9212,7 @@
       <c r="C79" s="36"/>
       <c r="D79" s="36"/>
       <c r="E79" s="38" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F79" s="38"/>
       <c r="G79" s="38"/>
@@ -9236,7 +9239,7 @@
       <c r="C80" s="36"/>
       <c r="D80" s="36"/>
       <c r="E80" s="38" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F80" s="38"/>
       <c r="G80" s="38"/>
@@ -9263,7 +9266,7 @@
       <c r="C81" s="36"/>
       <c r="D81" s="36"/>
       <c r="E81" s="38" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F81" s="38"/>
       <c r="G81" s="38"/>
@@ -9297,7 +9300,7 @@
       <c r="C82" s="36"/>
       <c r="D82" s="36"/>
       <c r="E82" s="56" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F82" s="56"/>
       <c r="G82" s="56"/>
@@ -9321,7 +9324,7 @@
     </row>
     <row r="84" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
@@ -9356,7 +9359,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="34" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C85" s="34"/>
       <c r="D85" s="34"/>
@@ -9391,7 +9394,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="34" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C86" s="34"/>
       <c r="D86" s="34"/>
@@ -9509,7 +9512,7 @@
       <c r="C89" s="36"/>
       <c r="D89" s="36"/>
       <c r="E89" s="37" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F89" s="37"/>
       <c r="G89" s="37"/>
@@ -9529,7 +9532,7 @@
       <c r="C90" s="36"/>
       <c r="D90" s="36"/>
       <c r="E90" s="38" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F90" s="38"/>
       <c r="G90" s="38"/>
@@ -9570,7 +9573,7 @@
       <c r="C91" s="36"/>
       <c r="D91" s="36"/>
       <c r="E91" s="38" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F91" s="38"/>
       <c r="G91" s="38"/>
@@ -9611,7 +9614,7 @@
       <c r="C92" s="36"/>
       <c r="D92" s="36"/>
       <c r="E92" s="38" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F92" s="38"/>
       <c r="G92" s="38"/>
@@ -9652,7 +9655,7 @@
       <c r="C93" s="36"/>
       <c r="D93" s="36"/>
       <c r="E93" s="56" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F93" s="56"/>
       <c r="G93" s="56"/>
@@ -9713,7 +9716,7 @@
       <c r="C95" s="36"/>
       <c r="D95" s="36"/>
       <c r="E95" s="38" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F95" s="38"/>
       <c r="G95" s="38"/>
@@ -9803,7 +9806,7 @@
       <c r="C98" s="36"/>
       <c r="D98" s="36"/>
       <c r="E98" s="38" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F98" s="38"/>
       <c r="G98" s="38"/>
@@ -9830,7 +9833,7 @@
       <c r="C99" s="36"/>
       <c r="D99" s="36"/>
       <c r="E99" s="38" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F99" s="38"/>
       <c r="G99" s="38"/>
@@ -9857,7 +9860,7 @@
       <c r="C100" s="36"/>
       <c r="D100" s="36"/>
       <c r="E100" s="56" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F100" s="56"/>
       <c r="G100" s="56"/>
@@ -9886,7 +9889,7 @@
       <c r="C101" s="36"/>
       <c r="D101" s="36"/>
       <c r="E101" s="37" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F101" s="37"/>
       <c r="G101" s="37"/>
@@ -9906,7 +9909,7 @@
       <c r="C102" s="36"/>
       <c r="D102" s="36"/>
       <c r="E102" s="38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F102" s="38"/>
       <c r="G102" s="38"/>
@@ -9933,7 +9936,7 @@
       <c r="C103" s="36"/>
       <c r="D103" s="36"/>
       <c r="E103" s="38" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F103" s="38"/>
       <c r="G103" s="38"/>
@@ -9960,7 +9963,7 @@
       <c r="C104" s="36"/>
       <c r="D104" s="36"/>
       <c r="E104" s="38" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F104" s="38"/>
       <c r="G104" s="38"/>
@@ -9987,7 +9990,7 @@
       <c r="C105" s="36"/>
       <c r="D105" s="36"/>
       <c r="E105" s="56" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F105" s="56"/>
       <c r="G105" s="56"/>
@@ -10014,7 +10017,7 @@
       <c r="C106" s="36"/>
       <c r="D106" s="36"/>
       <c r="E106" s="38" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F106" s="38"/>
       <c r="G106" s="38"/>
@@ -10068,7 +10071,7 @@
       <c r="C108" s="36"/>
       <c r="D108" s="36"/>
       <c r="E108" s="37" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F108" s="37"/>
       <c r="G108" s="37"/>
@@ -10088,7 +10091,7 @@
       <c r="C109" s="36"/>
       <c r="D109" s="36"/>
       <c r="E109" s="38" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F109" s="38"/>
       <c r="G109" s="38"/>
@@ -10115,7 +10118,7 @@
       <c r="C110" s="36"/>
       <c r="D110" s="36"/>
       <c r="E110" s="56" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F110" s="56"/>
       <c r="G110" s="56"/>
@@ -10142,7 +10145,7 @@
       <c r="C111" s="36"/>
       <c r="D111" s="36"/>
       <c r="E111" s="37" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F111" s="37"/>
       <c r="G111" s="37"/>
@@ -10162,7 +10165,7 @@
       <c r="C112" s="36"/>
       <c r="D112" s="36"/>
       <c r="E112" s="38" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F112" s="38"/>
       <c r="G112" s="38"/>
@@ -10186,12 +10189,12 @@
     </row>
     <row r="113" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B113" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C113" s="36"/>
       <c r="D113" s="36"/>
       <c r="E113" s="38" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F113" s="38"/>
       <c r="G113" s="38"/>
@@ -10245,7 +10248,7 @@
       <c r="C115" s="36"/>
       <c r="D115" s="36"/>
       <c r="E115" s="38" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F115" s="38"/>
       <c r="G115" s="38"/>
@@ -10272,7 +10275,7 @@
       <c r="C116" s="36"/>
       <c r="D116" s="36"/>
       <c r="E116" s="56" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F116" s="56"/>
       <c r="G116" s="56"/>
@@ -16266,7 +16269,7 @@
       <c r="S26" s="50"/>
       <c r="T26" s="50"/>
       <c r="U26" s="38" t="s">
-        <v>128</v>
+        <v>181</v>
       </c>
       <c r="V26" s="38"/>
       <c r="W26" s="38"/>
@@ -16287,7 +16290,7 @@
     </row>
     <row r="27" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -16316,7 +16319,7 @@
       <c r="S27" s="50"/>
       <c r="T27" s="50"/>
       <c r="U27" s="38" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="V27" s="38"/>
       <c r="W27" s="38"/>
@@ -16385,7 +16388,7 @@
     </row>
     <row r="32" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -16558,7 +16561,7 @@
       <c r="C37" s="36"/>
       <c r="D37" s="36"/>
       <c r="E37" s="38" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F37" s="38"/>
       <c r="G37" s="38"/>
@@ -16588,7 +16591,7 @@
       <c r="C38" s="36"/>
       <c r="D38" s="36"/>
       <c r="E38" s="37" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F38" s="37"/>
       <c r="G38" s="37"/>
@@ -16608,7 +16611,7 @@
       <c r="C39" s="36"/>
       <c r="D39" s="36"/>
       <c r="E39" s="38" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F39" s="38"/>
       <c r="G39" s="38"/>
@@ -16857,7 +16860,7 @@
     </row>
     <row r="6" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -16892,7 +16895,7 @@
     </row>
     <row r="7" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="20" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C7" s="20"/>
       <c r="D7" s="20"/>
@@ -16927,7 +16930,7 @@
     </row>
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="20" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C8" s="20"/>
       <c r="D8" s="20"/>
@@ -16962,7 +16965,7 @@
     </row>
     <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="20" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C9" s="20"/>
       <c r="D9" s="20"/>
@@ -16997,7 +17000,7 @@
     </row>
     <row r="10" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="20" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
@@ -17032,7 +17035,7 @@
     </row>
     <row r="12" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -17101,7 +17104,7 @@
     </row>
     <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="12" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
@@ -17135,7 +17138,7 @@
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
@@ -17169,7 +17172,7 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
@@ -17203,7 +17206,7 @@
     </row>
     <row r="18" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="20" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C18" s="20"/>
       <c r="D18" s="20"/>
@@ -17238,7 +17241,7 @@
     </row>
     <row r="19" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="20" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C19" s="20"/>
       <c r="D19" s="20"/>
@@ -17273,7 +17276,7 @@
     </row>
     <row r="20" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="20" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
@@ -17308,7 +17311,7 @@
     </row>
     <row r="22" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -17636,7 +17639,7 @@
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
@@ -17671,7 +17674,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="34" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C6" s="34"/>
       <c r="D6" s="34"/>
@@ -17727,7 +17730,7 @@
       <c r="S7" s="23"/>
       <c r="T7" s="23"/>
       <c r="U7" s="24" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="V7" s="24"/>
       <c r="W7" s="24"/>
@@ -17735,7 +17738,7 @@
       <c r="Y7" s="24"/>
       <c r="Z7" s="24"/>
       <c r="AA7" s="24" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AB7" s="24"/>
       <c r="AC7" s="24"/>
@@ -17745,7 +17748,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="30" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C8" s="30"/>
       <c r="D8" s="30"/>
@@ -17782,7 +17785,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="30" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C9" s="30"/>
       <c r="D9" s="30"/>
@@ -17819,7 +17822,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="30" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C10" s="30"/>
       <c r="D10" s="30"/>
@@ -17856,7 +17859,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="30" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
@@ -17893,7 +17896,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="30" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -17930,7 +17933,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C13" s="30"/>
       <c r="D13" s="30"/>
@@ -17967,7 +17970,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="30" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C14" s="30"/>
       <c r="D14" s="30"/>
@@ -18004,7 +18007,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="30" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C15" s="30"/>
       <c r="D15" s="30"/>
@@ -18041,7 +18044,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C16" s="30"/>
       <c r="D16" s="30"/>
@@ -18078,7 +18081,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C17" s="30"/>
       <c r="D17" s="30"/>
@@ -18115,7 +18118,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="30" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C18" s="30"/>
       <c r="D18" s="30"/>
@@ -18152,7 +18155,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="30" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
@@ -18189,7 +18192,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="30" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
@@ -18226,7 +18229,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="30" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
@@ -18300,7 +18303,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="30" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
@@ -18337,7 +18340,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="30" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
@@ -18374,7 +18377,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="30" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C25" s="30"/>
       <c r="D25" s="30"/>
@@ -18411,7 +18414,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="30" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C26" s="30"/>
       <c r="D26" s="30"/>
@@ -18448,7 +18451,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="30" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -18559,7 +18562,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="30" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C30" s="30"/>
       <c r="D30" s="30"/>
@@ -18596,7 +18599,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="30" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C31" s="30"/>
       <c r="D31" s="30"/>
@@ -18633,7 +18636,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="30" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C32" s="30"/>
       <c r="D32" s="30"/>
@@ -18670,7 +18673,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="30" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C33" s="30"/>
       <c r="D33" s="30"/>
@@ -18707,7 +18710,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="30" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C34" s="30"/>
       <c r="D34" s="30"/>
@@ -18744,7 +18747,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="30" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C35" s="30"/>
       <c r="D35" s="30"/>
@@ -18822,7 +18825,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C38" s="23"/>
       <c r="D38" s="23"/>
@@ -18856,7 +18859,7 @@
     </row>
     <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="12" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
@@ -18890,7 +18893,7 @@
     </row>
     <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="12" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
@@ -18924,7 +18927,7 @@
     </row>
     <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="12" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
@@ -18958,7 +18961,7 @@
     </row>
     <row r="42" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C42" s="12"/>
       <c r="D42" s="12"/>
@@ -18992,7 +18995,7 @@
     </row>
     <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="12" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
@@ -19026,7 +19029,7 @@
     </row>
     <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C44" s="12"/>
       <c r="D44" s="12"/>
@@ -19060,7 +19063,7 @@
     </row>
     <row r="45" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="12" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C45" s="12"/>
       <c r="D45" s="12"/>
@@ -19094,7 +19097,7 @@
     </row>
     <row r="46" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="12" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C46" s="12"/>
       <c r="D46" s="12"/>
@@ -19128,7 +19131,7 @@
     </row>
     <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="12" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C47" s="12"/>
       <c r="D47" s="12"/>
@@ -19162,7 +19165,7 @@
     </row>
     <row r="49" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
@@ -19197,7 +19200,7 @@
     </row>
     <row r="51" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -19232,7 +19235,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="34" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C52" s="34"/>
       <c r="D52" s="34"/>
@@ -19267,7 +19270,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="34" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C53" s="34"/>
       <c r="D53" s="34"/>
@@ -19346,7 +19349,7 @@
       <c r="C55" s="36"/>
       <c r="D55" s="36"/>
       <c r="E55" s="38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F55" s="38"/>
       <c r="G55" s="38"/>
@@ -19376,7 +19379,7 @@
       <c r="C56" s="36"/>
       <c r="D56" s="36"/>
       <c r="E56" s="38" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F56" s="38"/>
       <c r="G56" s="38"/>
@@ -19404,7 +19407,7 @@
       <c r="C57" s="36"/>
       <c r="D57" s="36"/>
       <c r="E57" s="38" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F57" s="38"/>
       <c r="G57" s="38"/>
@@ -19434,7 +19437,7 @@
       <c r="C58" s="36"/>
       <c r="D58" s="36"/>
       <c r="E58" s="37" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F58" s="37"/>
       <c r="G58" s="37"/>
@@ -19454,7 +19457,7 @@
       <c r="C59" s="36"/>
       <c r="D59" s="36"/>
       <c r="E59" s="38" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F59" s="38"/>
       <c r="G59" s="38"/>
@@ -19479,12 +19482,12 @@
     </row>
     <row r="60" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C60" s="36"/>
       <c r="D60" s="36"/>
       <c r="E60" s="38" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F60" s="38"/>
       <c r="G60" s="38"/>
@@ -19514,7 +19517,7 @@
       <c r="C61" s="36"/>
       <c r="D61" s="36"/>
       <c r="E61" s="38" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F61" s="38"/>
       <c r="G61" s="38"/>
@@ -19539,12 +19542,12 @@
     </row>
     <row r="62" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C62" s="36"/>
       <c r="D62" s="36"/>
       <c r="E62" s="38" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F62" s="38"/>
       <c r="G62" s="38"/>
@@ -19580,7 +19583,7 @@
       <c r="C63" s="36"/>
       <c r="D63" s="36"/>
       <c r="E63" s="38" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F63" s="38"/>
       <c r="G63" s="38"/>
@@ -19610,7 +19613,7 @@
       <c r="C64" s="36"/>
       <c r="D64" s="36"/>
       <c r="E64" s="38" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F64" s="38"/>
       <c r="G64" s="38"/>
@@ -19646,7 +19649,7 @@
       <c r="C65" s="36"/>
       <c r="D65" s="36"/>
       <c r="E65" s="56" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F65" s="56"/>
       <c r="G65" s="56"/>
@@ -19671,12 +19674,12 @@
     </row>
     <row r="66" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C66" s="36"/>
       <c r="D66" s="36"/>
       <c r="E66" s="37" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F66" s="37"/>
       <c r="G66" s="37"/>
@@ -19696,7 +19699,7 @@
       <c r="C67" s="36"/>
       <c r="D67" s="36"/>
       <c r="E67" s="38" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F67" s="38"/>
       <c r="G67" s="38"/>
@@ -19724,7 +19727,7 @@
       <c r="C68" s="36"/>
       <c r="D68" s="36"/>
       <c r="E68" s="38" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F68" s="38"/>
       <c r="G68" s="38"/>
@@ -19788,7 +19791,7 @@
       <c r="C70" s="36"/>
       <c r="D70" s="36"/>
       <c r="E70" s="37" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F70" s="37"/>
       <c r="G70" s="37"/>
@@ -19808,7 +19811,7 @@
       <c r="C71" s="36"/>
       <c r="D71" s="36"/>
       <c r="E71" s="38" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F71" s="38"/>
       <c r="G71" s="38"/>
@@ -19836,7 +19839,7 @@
       <c r="C72" s="36"/>
       <c r="D72" s="36"/>
       <c r="E72" s="38" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F72" s="38"/>
       <c r="G72" s="38"/>
@@ -19864,7 +19867,7 @@
       <c r="C73" s="36"/>
       <c r="D73" s="36"/>
       <c r="E73" s="38" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F73" s="38"/>
       <c r="G73" s="38"/>
@@ -19892,7 +19895,7 @@
       <c r="C74" s="36"/>
       <c r="D74" s="36"/>
       <c r="E74" s="38" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F74" s="38"/>
       <c r="G74" s="38"/>
@@ -19920,7 +19923,7 @@
       <c r="C75" s="36"/>
       <c r="D75" s="36"/>
       <c r="E75" s="38" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F75" s="38"/>
       <c r="G75" s="38"/>
@@ -19948,7 +19951,7 @@
       <c r="C76" s="36"/>
       <c r="D76" s="36"/>
       <c r="E76" s="38" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F76" s="38"/>
       <c r="G76" s="38"/>
@@ -20004,7 +20007,7 @@
       <c r="C78" s="36"/>
       <c r="D78" s="36"/>
       <c r="E78" s="38" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F78" s="38"/>
       <c r="G78" s="38"/>
@@ -20032,7 +20035,7 @@
       <c r="C79" s="36"/>
       <c r="D79" s="36"/>
       <c r="E79" s="38" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F79" s="38"/>
       <c r="G79" s="38"/>
@@ -20060,7 +20063,7 @@
       <c r="C80" s="36"/>
       <c r="D80" s="36"/>
       <c r="E80" s="38" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F80" s="38"/>
       <c r="G80" s="38"/>
@@ -20088,7 +20091,7 @@
       <c r="C81" s="36"/>
       <c r="D81" s="36"/>
       <c r="E81" s="38" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F81" s="38"/>
       <c r="G81" s="38"/>
@@ -20124,7 +20127,7 @@
       <c r="C82" s="36"/>
       <c r="D82" s="36"/>
       <c r="E82" s="56" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F82" s="56"/>
       <c r="G82" s="56"/>
@@ -20149,7 +20152,7 @@
     </row>
     <row r="84" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
@@ -20184,7 +20187,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B85" s="34" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C85" s="34"/>
       <c r="D85" s="34"/>
@@ -20219,7 +20222,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B86" s="34" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C86" s="34"/>
       <c r="D86" s="34"/>
@@ -20337,7 +20340,7 @@
       <c r="C89" s="36"/>
       <c r="D89" s="36"/>
       <c r="E89" s="37" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F89" s="37"/>
       <c r="G89" s="37"/>
@@ -20357,7 +20360,7 @@
       <c r="C90" s="36"/>
       <c r="D90" s="36"/>
       <c r="E90" s="38" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F90" s="38"/>
       <c r="G90" s="38"/>
@@ -20401,7 +20404,7 @@
       <c r="C91" s="36"/>
       <c r="D91" s="36"/>
       <c r="E91" s="38" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F91" s="38"/>
       <c r="G91" s="38"/>
@@ -20445,7 +20448,7 @@
       <c r="C92" s="36"/>
       <c r="D92" s="36"/>
       <c r="E92" s="38" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F92" s="38"/>
       <c r="G92" s="38"/>
@@ -20489,7 +20492,7 @@
       <c r="C93" s="36"/>
       <c r="D93" s="36"/>
       <c r="E93" s="56" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F93" s="56"/>
       <c r="G93" s="56"/>
@@ -20553,7 +20556,7 @@
       <c r="C95" s="36"/>
       <c r="D95" s="36"/>
       <c r="E95" s="38" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F95" s="38"/>
       <c r="G95" s="38"/>
@@ -20647,7 +20650,7 @@
       <c r="C98" s="36"/>
       <c r="D98" s="36"/>
       <c r="E98" s="38" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F98" s="38"/>
       <c r="G98" s="38"/>
@@ -20675,7 +20678,7 @@
       <c r="C99" s="36"/>
       <c r="D99" s="36"/>
       <c r="E99" s="38" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F99" s="38"/>
       <c r="G99" s="38"/>
@@ -20703,7 +20706,7 @@
       <c r="C100" s="36"/>
       <c r="D100" s="36"/>
       <c r="E100" s="56" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F100" s="56"/>
       <c r="G100" s="56"/>
@@ -20733,7 +20736,7 @@
       <c r="C101" s="36"/>
       <c r="D101" s="36"/>
       <c r="E101" s="37" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F101" s="37"/>
       <c r="G101" s="37"/>
@@ -20753,7 +20756,7 @@
       <c r="C102" s="36"/>
       <c r="D102" s="36"/>
       <c r="E102" s="38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F102" s="38"/>
       <c r="G102" s="38"/>
@@ -20781,7 +20784,7 @@
       <c r="C103" s="36"/>
       <c r="D103" s="36"/>
       <c r="E103" s="38" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F103" s="38"/>
       <c r="G103" s="38"/>
@@ -20809,7 +20812,7 @@
       <c r="C104" s="36"/>
       <c r="D104" s="36"/>
       <c r="E104" s="38" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F104" s="38"/>
       <c r="G104" s="38"/>
@@ -20837,7 +20840,7 @@
       <c r="C105" s="36"/>
       <c r="D105" s="36"/>
       <c r="E105" s="56" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F105" s="56"/>
       <c r="G105" s="56"/>
@@ -20865,7 +20868,7 @@
       <c r="C106" s="36"/>
       <c r="D106" s="36"/>
       <c r="E106" s="38" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F106" s="38"/>
       <c r="G106" s="38"/>
@@ -20921,7 +20924,7 @@
       <c r="C108" s="36"/>
       <c r="D108" s="36"/>
       <c r="E108" s="37" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F108" s="37"/>
       <c r="G108" s="37"/>
@@ -20941,7 +20944,7 @@
       <c r="C109" s="36"/>
       <c r="D109" s="36"/>
       <c r="E109" s="38" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F109" s="38"/>
       <c r="G109" s="38"/>
@@ -20969,7 +20972,7 @@
       <c r="C110" s="36"/>
       <c r="D110" s="36"/>
       <c r="E110" s="56" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F110" s="56"/>
       <c r="G110" s="56"/>
@@ -20997,7 +21000,7 @@
       <c r="C111" s="36"/>
       <c r="D111" s="36"/>
       <c r="E111" s="37" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F111" s="37"/>
       <c r="G111" s="37"/>
@@ -21017,7 +21020,7 @@
       <c r="C112" s="36"/>
       <c r="D112" s="36"/>
       <c r="E112" s="38" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F112" s="38"/>
       <c r="G112" s="38"/>
@@ -21042,12 +21045,12 @@
     </row>
     <row r="113" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B113" s="36" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C113" s="36"/>
       <c r="D113" s="36"/>
       <c r="E113" s="38" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F113" s="38"/>
       <c r="G113" s="38"/>
@@ -21103,7 +21106,7 @@
       <c r="C115" s="36"/>
       <c r="D115" s="36"/>
       <c r="E115" s="38" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F115" s="38"/>
       <c r="G115" s="38"/>
@@ -21131,7 +21134,7 @@
       <c r="C116" s="36"/>
       <c r="D116" s="36"/>
       <c r="E116" s="56" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F116" s="56"/>
       <c r="G116" s="56"/>
@@ -21501,7 +21504,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -21536,7 +21539,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -21571,7 +21574,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>

</xml_diff>